<commit_message>
Correcciones de la estructura de la base de datos
</commit_message>
<xml_diff>
--- a/documentacion/DD Proyecto.xlsx
+++ b/documentacion/DD Proyecto.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\52664\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shavi\Downloads\visual\Proyecto\RBE\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C467BFB1-A06E-4110-A3DD-D5BCE986FB8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E46209B4-BF96-48FD-8E7E-59C9A9130545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15360" yWindow="0" windowWidth="7776" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DICCIONARIO DE DATOS" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="140">
   <si>
     <t>Número</t>
   </si>
@@ -454,6 +454,12 @@
   </si>
   <si>
     <t>Es el numero que identifica el tipo de pago</t>
+  </si>
+  <si>
+    <t>VIAJE_ASIENTO</t>
+  </si>
+  <si>
+    <t>Asociar el estado de un asiento en un viaje especifico.</t>
   </si>
 </sst>
 </file>
@@ -884,19 +890,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A4:F149"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A4:F155"/>
+  <sheetFormatPr defaultColWidth="11.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.08984375" style="2"/>
-    <col min="2" max="2" width="16.6328125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.36328125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="11.08984375" style="2"/>
-    <col min="5" max="5" width="11.08984375" style="3"/>
-    <col min="6" max="6" width="33.36328125" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="11.08984375" style="2"/>
+    <col min="1" max="1" width="11.109375" style="2"/>
+    <col min="2" max="2" width="16.6640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" style="2"/>
+    <col min="5" max="5" width="11.109375" style="3"/>
+    <col min="6" max="6" width="33.33203125" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="11.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
         <v>75</v>
       </c>
@@ -904,7 +910,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
         <v>93</v>
       </c>
@@ -912,7 +918,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>0</v>
       </c>
@@ -932,7 +938,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="7">
         <v>1</v>
       </c>
@@ -950,7 +956,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="7">
         <v>2</v>
       </c>
@@ -970,7 +976,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="7">
         <v>3</v>
       </c>
@@ -988,7 +994,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="7">
         <v>4</v>
       </c>
@@ -1006,7 +1012,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="7">
         <v>5</v>
       </c>
@@ -1024,7 +1030,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="7">
         <v>6</v>
       </c>
@@ -1044,7 +1050,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
         <v>75</v>
       </c>
@@ -1052,7 +1058,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
         <v>93</v>
       </c>
@@ -1060,7 +1066,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>0</v>
       </c>
@@ -1080,7 +1086,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="7">
         <v>1</v>
       </c>
@@ -1096,7 +1102,7 @@
       </c>
       <c r="F17" s="8"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="7">
         <v>2</v>
       </c>
@@ -1116,7 +1122,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="7">
         <v>3</v>
       </c>
@@ -1136,7 +1142,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="7">
         <v>4</v>
       </c>
@@ -1154,7 +1160,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="7">
         <v>5</v>
       </c>
@@ -1174,7 +1180,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="7">
         <v>6</v>
       </c>
@@ -1192,7 +1198,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="7">
         <v>7</v>
       </c>
@@ -1210,7 +1216,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
         <v>75</v>
       </c>
@@ -1218,7 +1224,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
         <v>93</v>
       </c>
@@ -1226,7 +1232,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>0</v>
       </c>
@@ -1246,7 +1252,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="7">
         <v>1</v>
       </c>
@@ -1266,7 +1272,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="7">
         <v>2</v>
       </c>
@@ -1286,7 +1292,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="12" t="s">
         <v>75</v>
       </c>
@@ -1294,7 +1300,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="12" t="s">
         <v>93</v>
       </c>
@@ -1302,7 +1308,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>0</v>
       </c>
@@ -1322,7 +1328,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A34" s="7">
         <v>1</v>
       </c>
@@ -1342,7 +1348,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="7">
         <v>2</v>
       </c>
@@ -1362,7 +1368,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="12" t="s">
         <v>75</v>
       </c>
@@ -1370,7 +1376,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="12" t="s">
         <v>93</v>
       </c>
@@ -1378,7 +1384,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>0</v>
       </c>
@@ -1398,7 +1404,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="7">
         <v>1</v>
       </c>
@@ -1416,7 +1422,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="7">
         <v>2</v>
       </c>
@@ -1434,7 +1440,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="7">
         <v>3</v>
       </c>
@@ -1454,7 +1460,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="12" t="s">
         <v>75</v>
       </c>
@@ -1462,7 +1468,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="12" t="s">
         <v>93</v>
       </c>
@@ -1470,7 +1476,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
         <v>0</v>
       </c>
@@ -1490,7 +1496,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="7">
         <v>1</v>
       </c>
@@ -1508,7 +1514,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="7">
         <v>2</v>
       </c>
@@ -1526,7 +1532,7 @@
       </c>
       <c r="F48" s="9"/>
     </row>
-    <row r="49" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A49" s="7">
         <v>3</v>
       </c>
@@ -1544,7 +1550,7 @@
       </c>
       <c r="F49" s="9"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="12" t="s">
         <v>75</v>
       </c>
@@ -1552,7 +1558,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="12" t="s">
         <v>93</v>
       </c>
@@ -1560,7 +1566,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
         <v>0</v>
       </c>
@@ -1580,7 +1586,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="7">
         <v>1</v>
       </c>
@@ -1596,7 +1602,7 @@
       </c>
       <c r="F54" s="9"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="7">
         <v>2</v>
       </c>
@@ -1614,7 +1620,7 @@
       </c>
       <c r="F55" s="9"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="7">
         <v>3</v>
       </c>
@@ -1632,7 +1638,7 @@
       </c>
       <c r="F56" s="9"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="12" t="s">
         <v>75</v>
       </c>
@@ -1640,7 +1646,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="12" t="s">
         <v>93</v>
       </c>
@@ -1648,7 +1654,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
         <v>0</v>
       </c>
@@ -1668,7 +1674,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="7">
         <v>1</v>
       </c>
@@ -1684,7 +1690,7 @@
       </c>
       <c r="F61" s="9"/>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="7">
         <v>2</v>
       </c>
@@ -1702,7 +1708,7 @@
       </c>
       <c r="F62" s="9"/>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="7">
         <v>3</v>
       </c>
@@ -1720,7 +1726,7 @@
       </c>
       <c r="F63" s="9"/>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="7">
         <v>4</v>
       </c>
@@ -1738,7 +1744,7 @@
       </c>
       <c r="F64" s="9"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="7">
         <v>5</v>
       </c>
@@ -1756,7 +1762,7 @@
       </c>
       <c r="F65" s="9"/>
     </row>
-    <row r="66" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A66" s="7">
         <v>6</v>
       </c>
@@ -1774,7 +1780,7 @@
       </c>
       <c r="F66" s="9"/>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="12" t="s">
         <v>75</v>
       </c>
@@ -1782,7 +1788,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="12" t="s">
         <v>93</v>
       </c>
@@ -1790,7 +1796,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
         <v>0</v>
       </c>
@@ -1810,7 +1816,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A71" s="7">
         <v>1</v>
       </c>
@@ -1828,7 +1834,7 @@
       </c>
       <c r="F71" s="9"/>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="7">
         <v>2</v>
       </c>
@@ -1846,7 +1852,7 @@
       </c>
       <c r="F72" s="9"/>
     </row>
-    <row r="73" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A73" s="7">
         <v>3</v>
       </c>
@@ -1862,7 +1868,7 @@
       </c>
       <c r="F73" s="9"/>
     </row>
-    <row r="74" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A74" s="7">
         <v>4</v>
       </c>
@@ -1878,7 +1884,7 @@
       </c>
       <c r="F74" s="9"/>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="12" t="s">
         <v>75</v>
       </c>
@@ -1886,7 +1892,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="12" t="s">
         <v>93</v>
       </c>
@@ -1894,7 +1900,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
         <v>0</v>
       </c>
@@ -1914,7 +1920,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="79" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A79" s="7">
         <v>1</v>
       </c>
@@ -1930,7 +1936,7 @@
       </c>
       <c r="F79" s="9"/>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="7">
         <v>2</v>
       </c>
@@ -1946,7 +1952,7 @@
       </c>
       <c r="F80" s="9"/>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="7">
         <v>3</v>
       </c>
@@ -1962,7 +1968,7 @@
       </c>
       <c r="F81" s="9"/>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="7">
         <v>4</v>
       </c>
@@ -1978,7 +1984,7 @@
       </c>
       <c r="F82" s="9"/>
     </row>
-    <row r="83" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A83" s="7">
         <v>5</v>
       </c>
@@ -1996,7 +2002,7 @@
       </c>
       <c r="F83" s="9"/>
     </row>
-    <row r="84" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A84" s="7">
         <v>6</v>
       </c>
@@ -2012,7 +2018,7 @@
       </c>
       <c r="F84" s="9"/>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="12" t="s">
         <v>75</v>
       </c>
@@ -2020,7 +2026,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="12" t="s">
         <v>93</v>
       </c>
@@ -2028,7 +2034,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="5" t="s">
         <v>0</v>
       </c>
@@ -2048,7 +2054,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="7">
         <v>1</v>
       </c>
@@ -2064,7 +2070,7 @@
       </c>
       <c r="F89" s="8"/>
     </row>
-    <row r="90" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A90" s="7">
         <v>2</v>
       </c>
@@ -2082,7 +2088,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="91" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A91" s="7">
         <v>3</v>
       </c>
@@ -2102,7 +2108,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="12" t="s">
         <v>75</v>
       </c>
@@ -2110,7 +2116,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="12" t="s">
         <v>93</v>
       </c>
@@ -2118,7 +2124,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
         <v>0</v>
       </c>
@@ -2138,7 +2144,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="7">
         <v>1</v>
       </c>
@@ -2154,7 +2160,7 @@
       </c>
       <c r="F96" s="9"/>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="7">
         <v>2</v>
       </c>
@@ -2170,7 +2176,7 @@
       </c>
       <c r="F97" s="9"/>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="7">
         <v>3</v>
       </c>
@@ -2186,7 +2192,7 @@
       </c>
       <c r="F98" s="9"/>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="12" t="s">
         <v>75</v>
       </c>
@@ -2194,7 +2200,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="12" t="s">
         <v>93</v>
       </c>
@@ -2202,7 +2208,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
         <v>0</v>
       </c>
@@ -2222,7 +2228,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="103" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A103" s="7">
         <v>1</v>
       </c>
@@ -2240,7 +2246,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="104" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A104" s="7">
         <v>2</v>
       </c>
@@ -2258,7 +2264,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="105" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A105" s="7">
         <v>3</v>
       </c>
@@ -2276,7 +2282,7 @@
       </c>
       <c r="F105" s="9"/>
     </row>
-    <row r="106" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A106" s="7">
         <v>4</v>
       </c>
@@ -2292,7 +2298,7 @@
       </c>
       <c r="F106" s="9"/>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" s="12" t="s">
         <v>75</v>
       </c>
@@ -2300,7 +2306,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="12" t="s">
         <v>93</v>
       </c>
@@ -2308,7 +2314,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
         <v>0</v>
       </c>
@@ -2328,7 +2334,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="111" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A111" s="7">
         <v>1</v>
       </c>
@@ -2344,7 +2350,7 @@
       </c>
       <c r="F111" s="9"/>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="7">
         <v>2</v>
       </c>
@@ -2362,7 +2368,7 @@
       </c>
       <c r="F112" s="9"/>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="7">
         <v>3</v>
       </c>
@@ -2380,7 +2386,7 @@
       </c>
       <c r="F113" s="9"/>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="7">
         <v>4</v>
       </c>
@@ -2396,7 +2402,7 @@
       <c r="E114" s="8"/>
       <c r="F114" s="9"/>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="7">
         <v>5</v>
       </c>
@@ -2412,7 +2418,7 @@
       </c>
       <c r="F115" s="9"/>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="7">
         <v>6</v>
       </c>
@@ -2426,7 +2432,7 @@
       <c r="E116" s="8"/>
       <c r="F116" s="9"/>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="12" t="s">
         <v>75</v>
       </c>
@@ -2434,7 +2440,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="12" t="s">
         <v>93</v>
       </c>
@@ -2442,7 +2448,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="5" t="s">
         <v>0</v>
       </c>
@@ -2462,7 +2468,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="121" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A121" s="7">
         <v>1</v>
       </c>
@@ -2480,7 +2486,7 @@
       </c>
       <c r="F121" s="9"/>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="7">
         <v>2</v>
       </c>
@@ -2496,7 +2502,7 @@
       </c>
       <c r="F122" s="9"/>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="7">
         <v>3</v>
       </c>
@@ -2512,7 +2518,7 @@
       </c>
       <c r="F123" s="9"/>
     </row>
-    <row r="124" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A124" s="7">
         <v>4</v>
       </c>
@@ -2528,7 +2534,7 @@
       </c>
       <c r="F124" s="9"/>
     </row>
-    <row r="125" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A125" s="7">
         <v>5</v>
       </c>
@@ -2544,7 +2550,7 @@
       </c>
       <c r="F125" s="9"/>
     </row>
-    <row r="126" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A126" s="7">
         <v>6</v>
       </c>
@@ -2560,7 +2566,7 @@
       </c>
       <c r="F126" s="9"/>
     </row>
-    <row r="127" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A127" s="7">
         <v>7</v>
       </c>
@@ -2576,7 +2582,7 @@
       </c>
       <c r="F127" s="9"/>
     </row>
-    <row r="128" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A128" s="7">
         <v>8</v>
       </c>
@@ -2594,7 +2600,7 @@
       </c>
       <c r="F128" s="9"/>
     </row>
-    <row r="129" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A129" s="7">
         <v>9</v>
       </c>
@@ -2610,7 +2616,7 @@
       </c>
       <c r="F129" s="9"/>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="12" t="s">
         <v>75</v>
       </c>
@@ -2618,7 +2624,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" s="12" t="s">
         <v>93</v>
       </c>
@@ -2626,7 +2632,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" s="5" t="s">
         <v>0</v>
       </c>
@@ -2646,7 +2652,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="134" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A134" s="7">
         <v>1</v>
       </c>
@@ -2664,7 +2670,7 @@
       </c>
       <c r="F134" s="9"/>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" s="7">
         <v>2</v>
       </c>
@@ -2680,7 +2686,7 @@
       </c>
       <c r="F135" s="9"/>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" s="7">
         <v>3</v>
       </c>
@@ -2696,7 +2702,7 @@
       </c>
       <c r="F136" s="9"/>
     </row>
-    <row r="137" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A137" s="7">
         <v>4</v>
       </c>
@@ -2712,7 +2718,7 @@
       </c>
       <c r="F137" s="9"/>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" s="12" t="s">
         <v>75</v>
       </c>
@@ -2720,7 +2726,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" s="12" t="s">
         <v>93</v>
       </c>
@@ -2728,7 +2734,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" s="5" t="s">
         <v>0</v>
       </c>
@@ -2748,7 +2754,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" s="7">
         <v>1</v>
       </c>
@@ -2764,7 +2770,7 @@
       </c>
       <c r="F142" s="9"/>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" s="7">
         <v>2</v>
       </c>
@@ -2782,7 +2788,7 @@
       </c>
       <c r="F143" s="9"/>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" s="7">
         <v>3</v>
       </c>
@@ -2800,7 +2806,7 @@
       </c>
       <c r="F144" s="9"/>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" s="7">
         <v>4</v>
       </c>
@@ -2816,7 +2822,7 @@
       <c r="E145" s="8"/>
       <c r="F145" s="9"/>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" s="7">
         <v>5</v>
       </c>
@@ -2832,7 +2838,7 @@
       </c>
       <c r="F146" s="9"/>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" s="7">
         <v>6</v>
       </c>
@@ -2850,7 +2856,7 @@
       </c>
       <c r="F147" s="9"/>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" s="7">
         <v>7</v>
       </c>
@@ -2868,7 +2874,7 @@
       </c>
       <c r="F148" s="9"/>
     </row>
-    <row r="149" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A149" s="7">
         <v>8</v>
       </c>
@@ -2883,6 +2889,74 @@
         <v>72</v>
       </c>
       <c r="F149" s="9"/>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A151" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B151" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A152" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B152" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A153" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B153" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C153" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D153" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E153" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F153" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A154" s="7">
+        <v>1</v>
+      </c>
+      <c r="B154" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C154" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D154" s="7"/>
+      <c r="E154" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F154" s="9"/>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A155" s="7">
+        <v>2</v>
+      </c>
+      <c r="B155" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C155" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D155" s="7"/>
+      <c r="E155" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F155" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
actualice la tabla ruta
</commit_message>
<xml_diff>
--- a/documentacion/DD Proyecto.xlsx
+++ b/documentacion/DD Proyecto.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\52664\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shavi\Downloads\visual\Proyecto\RBE\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4815E627-5002-46DB-B3AA-B5AD56A6A790}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D90EE08-E5EB-494B-A85F-3FC8EE9526D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DICCIONARIO DE DATOS" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'DICCIONARIO DE DATOS'!$A$1:$F$156</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'DICCIONARIO DE DATOS'!$A$1:$F$157</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="201">
   <si>
     <t>Número</t>
   </si>
@@ -632,6 +632,19 @@
   </si>
   <si>
     <t>Almacena las marcas de los autobuses registrados en la empresa.</t>
+  </si>
+  <si>
+    <t>costo</t>
+  </si>
+  <si>
+    <t>decimal</t>
+  </si>
+  <si>
+    <t>NOT NULL
+DEFAULT</t>
+  </si>
+  <si>
+    <t>Es el coste de la ruta por ticket para luego calcular el costo del ticket, con valor por defecto de 250</t>
   </si>
 </sst>
 </file>
@@ -1062,19 +1075,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A4:G156"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A4:G157"/>
+  <sheetFormatPr defaultColWidth="11.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.08984375" style="2"/>
-    <col min="2" max="2" width="16.6328125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="16.1796875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.1796875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="12.90625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="33.36328125" style="12" customWidth="1"/>
-    <col min="7" max="16384" width="11.08984375" style="2"/>
+    <col min="1" max="1" width="11.109375" style="2"/>
+    <col min="2" max="2" width="16.6640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="16.21875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="12.21875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="33.33203125" style="12" customWidth="1"/>
+    <col min="7" max="16384" width="11.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>66</v>
       </c>
@@ -1082,7 +1095,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>83</v>
       </c>
@@ -1090,7 +1103,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>0</v>
       </c>
@@ -1110,7 +1123,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>1</v>
       </c>
@@ -1128,7 +1141,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="6">
         <v>2</v>
       </c>
@@ -1151,7 +1164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
         <v>66</v>
       </c>
@@ -1159,7 +1172,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>83</v>
       </c>
@@ -1167,7 +1180,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>0</v>
       </c>
@@ -1187,7 +1200,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>1</v>
       </c>
@@ -1205,7 +1218,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="6">
         <v>2</v>
       </c>
@@ -1225,7 +1238,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>3</v>
       </c>
@@ -1245,7 +1258,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="6">
         <v>4</v>
       </c>
@@ -1263,7 +1276,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>5</v>
       </c>
@@ -1283,7 +1296,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="6">
         <v>6</v>
       </c>
@@ -1301,7 +1314,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>7</v>
       </c>
@@ -1322,7 +1335,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
         <v>66</v>
       </c>
@@ -1330,7 +1343,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
         <v>83</v>
       </c>
@@ -1338,7 +1351,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>0</v>
       </c>
@@ -1358,7 +1371,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="6">
         <v>1</v>
       </c>
@@ -1378,7 +1391,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>2</v>
       </c>
@@ -1401,7 +1414,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="10" t="s">
         <v>66</v>
       </c>
@@ -1409,7 +1422,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
         <v>83</v>
       </c>
@@ -1417,7 +1430,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>0</v>
       </c>
@@ -1437,7 +1450,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="6">
         <v>1</v>
       </c>
@@ -1457,7 +1470,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="6">
         <v>2</v>
       </c>
@@ -1480,7 +1493,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="10" t="s">
         <v>66</v>
       </c>
@@ -1488,7 +1501,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="10" t="s">
         <v>83</v>
       </c>
@@ -1496,7 +1509,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>0</v>
       </c>
@@ -1516,7 +1529,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A36" s="6">
         <v>1</v>
       </c>
@@ -1534,7 +1547,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="6">
         <v>2</v>
       </c>
@@ -1552,7 +1565,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38" s="6">
         <v>3</v>
       </c>
@@ -1575,7 +1588,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="10" t="s">
         <v>66</v>
       </c>
@@ -1583,7 +1596,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="10" t="s">
         <v>83</v>
       </c>
@@ -1591,7 +1604,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>0</v>
       </c>
@@ -1611,7 +1624,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="6">
         <v>1</v>
       </c>
@@ -1629,7 +1642,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="6">
         <v>2</v>
       </c>
@@ -1649,7 +1662,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A45" s="6">
         <v>3</v>
       </c>
@@ -1672,7 +1685,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="10" t="s">
         <v>66</v>
       </c>
@@ -1680,7 +1693,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="10" t="s">
         <v>83</v>
       </c>
@@ -1688,7 +1701,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
         <v>0</v>
       </c>
@@ -1708,7 +1721,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="6">
         <v>1</v>
       </c>
@@ -1726,7 +1739,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="6">
         <v>2</v>
       </c>
@@ -1746,7 +1759,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A52" s="6">
         <v>3</v>
       </c>
@@ -1764,7 +1777,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A53" s="6">
         <v>4</v>
       </c>
@@ -1782,7 +1795,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A54" s="6">
         <v>5</v>
       </c>
@@ -1800,7 +1813,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A55" s="6">
         <v>6</v>
       </c>
@@ -1821,7 +1834,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="10" t="s">
         <v>66</v>
       </c>
@@ -1829,7 +1842,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="10" t="s">
         <v>83</v>
       </c>
@@ -1837,7 +1850,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
         <v>0</v>
       </c>
@@ -1857,7 +1870,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A60" s="6">
         <v>1</v>
       </c>
@@ -1875,7 +1888,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="6">
         <v>2</v>
       </c>
@@ -1895,7 +1908,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="62" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A62" s="6">
         <v>3</v>
       </c>
@@ -1918,7 +1931,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="10" t="s">
         <v>66</v>
       </c>
@@ -1926,7 +1939,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" s="10" t="s">
         <v>83</v>
       </c>
@@ -1934,7 +1947,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>0</v>
       </c>
@@ -1954,7 +1967,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="6">
         <v>1</v>
       </c>
@@ -1972,7 +1985,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" s="6">
         <v>2</v>
       </c>
@@ -1992,7 +2005,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="6">
         <v>3</v>
       </c>
@@ -2012,7 +2025,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A70" s="6">
         <v>4</v>
       </c>
@@ -2032,7 +2045,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="71" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A71" s="6">
         <v>5</v>
       </c>
@@ -2043,7 +2056,7 @@
         <v>61</v>
       </c>
       <c r="D71" s="6">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E71" s="7" t="s">
         <v>64</v>
@@ -2052,127 +2065,129 @@
         <v>152</v>
       </c>
     </row>
-    <row r="72" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A72" s="6">
         <v>6</v>
       </c>
       <c r="B72" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="D72" s="6">
+        <v>30</v>
+      </c>
+      <c r="E72" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="F72" s="11" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A73" s="6">
+        <v>7</v>
+      </c>
+      <c r="B73" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C72" s="6" t="s">
+      <c r="C73" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D72" s="6">
+      <c r="D73" s="6">
         <v>5</v>
       </c>
-      <c r="E72" s="7" t="s">
+      <c r="E73" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="F72" s="11" t="s">
+      <c r="F73" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="G72" s="2">
+      <c r="G73" s="2">
         <v>9</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A74" s="10" t="s">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A75" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B74" s="1" t="s">
+      <c r="B75" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A75" s="10" t="s">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A76" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="B76" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A76" s="4" t="s">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A77" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B76" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C76" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D76" s="4" t="s">
+      <c r="B77" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D77" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E76" s="5" t="s">
+      <c r="E77" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F76" s="5" t="s">
+      <c r="F77" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="77" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A77" s="6">
-        <v>1</v>
-      </c>
-      <c r="B77" s="6" t="s">
+    <row r="78" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A78" s="6">
+        <v>1</v>
+      </c>
+      <c r="B78" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C77" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D77" s="6"/>
-      <c r="E77" s="7" t="s">
+      <c r="C78" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D78" s="6"/>
+      <c r="E78" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="F77" s="11" t="s">
+      <c r="F78" s="11" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A78" s="6">
-        <v>2</v>
-      </c>
-      <c r="B78" s="6" t="s">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A79" s="6">
+        <v>2</v>
+      </c>
+      <c r="B79" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C78" s="6" t="s">
+      <c r="C79" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D78" s="6">
+      <c r="D79" s="6">
         <v>10</v>
       </c>
-      <c r="E78" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="F78" s="11" t="s">
+      <c r="E79" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="F79" s="11" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="79" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A79" s="6">
+    <row r="80" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A80" s="6">
         <v>3</v>
       </c>
-      <c r="B79" s="6" t="s">
+      <c r="B80" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="C79" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D79" s="6"/>
-      <c r="E79" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="F79" s="11" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A80" s="6">
-        <v>4</v>
-      </c>
-      <c r="B80" s="6" t="s">
-        <v>27</v>
       </c>
       <c r="C80" s="6" t="s">
         <v>59</v>
@@ -2182,90 +2197,90 @@
         <v>63</v>
       </c>
       <c r="F80" s="11" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A81" s="6">
+        <v>4</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D81" s="6"/>
+      <c r="E81" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F81" s="11" t="s">
         <v>158</v>
       </c>
-      <c r="G80" s="2">
+      <c r="G81" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A82" s="10" t="s">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A83" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B82" s="1" t="s">
+      <c r="B83" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A83" s="10" t="s">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A84" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B83" s="1" t="s">
+      <c r="B84" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A84" s="4" t="s">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A85" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B84" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C84" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D84" s="4" t="s">
+      <c r="B85" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D85" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E84" s="5" t="s">
+      <c r="E85" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F84" s="5" t="s">
+      <c r="F85" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="85" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A85" s="6">
-        <v>1</v>
-      </c>
-      <c r="B85" s="6" t="s">
+    <row r="86" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A86" s="6">
+        <v>1</v>
+      </c>
+      <c r="B86" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C85" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D85" s="6"/>
-      <c r="E85" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="F85" s="11" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A86" s="6">
-        <v>2</v>
-      </c>
-      <c r="B86" s="6" t="s">
-        <v>125</v>
-      </c>
       <c r="C86" s="6" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="D86" s="6"/>
       <c r="E86" s="7" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="F86" s="11" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C87" s="6" t="s">
         <v>101</v>
@@ -2275,33 +2290,33 @@
         <v>64</v>
       </c>
       <c r="F87" s="11" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>29</v>
+        <v>126</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>59</v>
+        <v>101</v>
       </c>
       <c r="D88" s="6"/>
       <c r="E88" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F88" s="11" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A89" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C89" s="6" t="s">
         <v>59</v>
@@ -2311,18 +2326,15 @@
         <v>63</v>
       </c>
       <c r="F89" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="G89" s="2">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A90" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C90" s="6" t="s">
         <v>59</v>
@@ -2332,15 +2344,18 @@
         <v>63</v>
       </c>
       <c r="F90" s="11" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>165</v>
+      </c>
+      <c r="G90" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A91" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C91" s="6" t="s">
         <v>59</v>
@@ -2350,279 +2365,279 @@
         <v>63</v>
       </c>
       <c r="F91" s="11" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A92" s="6">
+        <v>7</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D92" s="6"/>
+      <c r="E92" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F92" s="11" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A93" s="10" t="s">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A94" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B93" s="1" t="s">
+      <c r="B94" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A94" s="10" t="s">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A95" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B94" s="1" t="s">
+      <c r="B95" s="1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A95" s="4" t="s">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A96" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B95" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C95" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D95" s="4" t="s">
+      <c r="B96" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D96" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E95" s="5" t="s">
+      <c r="E96" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F95" s="5" t="s">
+      <c r="F96" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="96" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A96" s="6">
-        <v>1</v>
-      </c>
-      <c r="B96" s="6" t="s">
+    <row r="97" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A97" s="6">
+        <v>1</v>
+      </c>
+      <c r="B97" s="6" t="s">
         <v>6</v>
-      </c>
-      <c r="C96" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D96" s="6"/>
-      <c r="E96" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F96" s="11" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A97" s="6">
-        <v>2</v>
-      </c>
-      <c r="B97" s="6" t="s">
-        <v>31</v>
       </c>
       <c r="C97" s="6" t="s">
         <v>59</v>
       </c>
       <c r="D97" s="6"/>
       <c r="E97" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F97" s="11" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A98" s="6">
+        <v>2</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D98" s="6"/>
+      <c r="E98" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="F97" s="11" t="s">
+      <c r="F98" s="11" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="98" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A98" s="6">
+    <row r="99" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A99" s="6">
         <v>3</v>
       </c>
-      <c r="B98" s="6" t="s">
+      <c r="B99" s="6" t="s">
         <v>32</v>
-      </c>
-      <c r="C98" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="D98" s="6">
-        <v>10</v>
-      </c>
-      <c r="E98" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="F98" s="11" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A99" s="6">
-        <v>4</v>
-      </c>
-      <c r="B99" s="6" t="s">
-        <v>127</v>
       </c>
       <c r="C99" s="6" t="s">
         <v>61</v>
       </c>
       <c r="D99" s="6">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E99" s="7" t="s">
         <v>65</v>
       </c>
       <c r="F99" s="11" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A100" s="6">
+        <v>4</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D100" s="6">
+        <v>17</v>
+      </c>
+      <c r="E100" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F100" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="G99" s="2">
+      <c r="G100" s="2">
         <v>12</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A101" s="10" t="s">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A102" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B101" s="1" t="s">
+      <c r="B102" s="1" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A102" s="10" t="s">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A103" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B102" s="1" t="s">
+      <c r="B103" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A103" s="4" t="s">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A104" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B103" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C103" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D103" s="4" t="s">
+      <c r="B104" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C104" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D104" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E103" s="5" t="s">
+      <c r="E104" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F103" s="5" t="s">
+      <c r="F104" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="104" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A104" s="6">
-        <v>1</v>
-      </c>
-      <c r="B104" s="6" t="s">
+    <row r="105" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A105" s="6">
+        <v>1</v>
+      </c>
+      <c r="B105" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C104" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D104" s="6"/>
-      <c r="E104" s="7" t="s">
+      <c r="C105" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D105" s="6"/>
+      <c r="E105" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="F104" s="11" t="s">
+      <c r="F105" s="11" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="105" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A105" s="6">
-        <v>2</v>
-      </c>
-      <c r="B105" s="6" t="s">
+    <row r="106" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A106" s="6">
+        <v>2</v>
+      </c>
+      <c r="B106" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C105" s="8" t="s">
+      <c r="C106" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="D105" s="6">
+      <c r="D106" s="6">
         <v>5</v>
       </c>
-      <c r="E105" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="F105" s="11" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A106" s="6">
-        <v>3</v>
-      </c>
-      <c r="B106" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C106" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D106" s="6"/>
       <c r="E106" s="7" t="s">
         <v>63</v>
       </c>
       <c r="F106" s="11" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A107" s="6">
+        <v>3</v>
+      </c>
+      <c r="B107" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C107" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D107" s="6"/>
+      <c r="E107" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F107" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="G106" s="2">
+      <c r="G107" s="2">
         <v>13</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A108" s="10" t="s">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A109" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B108" s="1" t="s">
+      <c r="B109" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A109" s="10" t="s">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A110" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B109" s="1" t="s">
+      <c r="B110" s="1" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A110" s="4" t="s">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A111" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B110" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C110" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D110" s="4" t="s">
+      <c r="B111" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D111" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E110" s="5" t="s">
+      <c r="E111" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F110" s="5" t="s">
+      <c r="F111" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="111" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A111" s="6">
-        <v>1</v>
-      </c>
-      <c r="B111" s="6" t="s">
+    <row r="112" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A112" s="6">
+        <v>1</v>
+      </c>
+      <c r="B112" s="6" t="s">
         <v>46</v>
-      </c>
-      <c r="C111" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D111" s="6"/>
-      <c r="E111" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="F111" s="11" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="112" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A112" s="6">
-        <v>2</v>
-      </c>
-      <c r="B112" s="6" t="s">
-        <v>35</v>
       </c>
       <c r="C112" s="6" t="s">
         <v>59</v>
@@ -2632,110 +2647,108 @@
         <v>34</v>
       </c>
       <c r="F112" s="11" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A113" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C113" s="6" t="s">
-        <v>128</v>
+        <v>59</v>
       </c>
       <c r="D113" s="6"/>
       <c r="E113" s="7" t="s">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="F113" s="11" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A114" s="6">
+        <v>3</v>
+      </c>
+      <c r="B114" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C114" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D114" s="6"/>
+      <c r="E114" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="F114" s="11" t="s">
         <v>173</v>
       </c>
-      <c r="G113" s="2">
+      <c r="G114" s="2">
         <v>14</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A115" s="10" t="s">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A116" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B115" s="1" t="s">
+      <c r="B116" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A116" s="10" t="s">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A117" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B116" s="1" t="s">
+      <c r="B117" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A117" s="4" t="s">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A118" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B117" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C117" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D117" s="4" t="s">
+      <c r="B118" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C118" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D118" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E117" s="5" t="s">
+      <c r="E118" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F117" s="5" t="s">
+      <c r="F118" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="118" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A118" s="6">
-        <v>1</v>
-      </c>
-      <c r="B118" s="6" t="s">
+    <row r="119" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A119" s="6">
+        <v>1</v>
+      </c>
+      <c r="B119" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C118" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D118" s="6"/>
-      <c r="E118" s="7" t="s">
+      <c r="C119" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D119" s="6"/>
+      <c r="E119" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="F118" s="11" t="s">
+      <c r="F119" s="11" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A119" s="6">
-        <v>2</v>
-      </c>
-      <c r="B119" s="6" t="s">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A120" s="6">
+        <v>2</v>
+      </c>
+      <c r="B120" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="C119" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="D119" s="6">
-        <v>30</v>
-      </c>
-      <c r="E119" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="F119" s="11" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A120" s="6">
-        <v>3</v>
-      </c>
-      <c r="B120" s="6" t="s">
-        <v>40</v>
       </c>
       <c r="C120" s="6" t="s">
         <v>61</v>
@@ -2747,15 +2760,15 @@
         <v>64</v>
       </c>
       <c r="F120" s="11" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A121" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B121" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C121" s="6" t="s">
         <v>61</v>
@@ -2763,162 +2776,164 @@
       <c r="D121" s="6">
         <v>30</v>
       </c>
-      <c r="E121" s="7"/>
+      <c r="E121" s="7" t="s">
+        <v>64</v>
+      </c>
       <c r="F121" s="11" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A122" s="6">
+        <v>4</v>
+      </c>
+      <c r="B122" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C122" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D122" s="6">
+        <v>30</v>
+      </c>
+      <c r="E122" s="7"/>
+      <c r="F122" s="11" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A122" s="6">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A123" s="6">
         <v>5</v>
       </c>
-      <c r="B122" s="6" t="s">
+      <c r="B123" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="C122" s="6" t="s">
+      <c r="C123" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D122" s="6"/>
-      <c r="E122" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="F122" s="11" t="s">
+      <c r="D123" s="6"/>
+      <c r="E123" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="F123" s="11" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A123" s="6">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A124" s="6">
         <v>6</v>
       </c>
-      <c r="B123" s="6" t="s">
+      <c r="B124" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C123" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D123" s="6"/>
-      <c r="E123" s="7"/>
-      <c r="F123" s="11" t="s">
+      <c r="C124" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D124" s="6"/>
+      <c r="E124" s="7"/>
+      <c r="F124" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="G123" s="2">
+      <c r="G124" s="2">
         <v>15</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A125" s="10" t="s">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A126" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B125" s="1" t="s">
+      <c r="B126" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A126" s="10" t="s">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A127" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B126" s="1" t="s">
+      <c r="B127" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A127" s="4" t="s">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A128" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B127" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C127" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D127" s="4" t="s">
+      <c r="B128" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D128" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E127" s="5" t="s">
+      <c r="E128" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F127" s="5" t="s">
+      <c r="F128" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="128" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A128" s="6">
-        <v>1</v>
-      </c>
-      <c r="B128" s="6" t="s">
+    <row r="129" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A129" s="6">
+        <v>1</v>
+      </c>
+      <c r="B129" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C128" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D128" s="6"/>
-      <c r="E128" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="F128" s="11" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A129" s="6">
-        <v>2</v>
-      </c>
-      <c r="B129" s="6" t="s">
-        <v>51</v>
-      </c>
       <c r="C129" s="6" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="D129" s="6"/>
       <c r="E129" s="7" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="F129" s="11" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A130" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B130" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C130" s="6" t="s">
-        <v>60</v>
+        <v>101</v>
       </c>
       <c r="D130" s="6"/>
       <c r="E130" s="7" t="s">
         <v>64</v>
       </c>
       <c r="F130" s="11" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="131" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A131" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B131" s="6" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="C131" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D131" s="6"/>
       <c r="E131" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F131" s="11" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="132" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A132" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B132" s="6" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="C132" s="6" t="s">
         <v>59</v>
@@ -2928,126 +2943,126 @@
         <v>63</v>
       </c>
       <c r="F132" s="11" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A133" s="6">
+        <v>5</v>
+      </c>
+      <c r="B133" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C133" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D133" s="6"/>
+      <c r="E133" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F133" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="G132" s="2">
+      <c r="G133" s="2">
         <v>16</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A134" s="10" t="s">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A135" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B134" s="1" t="s">
+      <c r="B135" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A135" s="10" t="s">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A136" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B135" s="1" t="s">
+      <c r="B136" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A136" s="4" t="s">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A137" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B136" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C136" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D136" s="4" t="s">
+      <c r="B137" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D137" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E136" s="5" t="s">
+      <c r="E137" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F136" s="5" t="s">
+      <c r="F137" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A137" s="6">
-        <v>1</v>
-      </c>
-      <c r="B137" s="6" t="s">
+    <row r="138" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A138" s="6">
+        <v>1</v>
+      </c>
+      <c r="B138" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C137" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D137" s="6"/>
-      <c r="E137" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="F137" s="11" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A138" s="6">
-        <v>2</v>
-      </c>
-      <c r="B138" s="6" t="s">
-        <v>44</v>
-      </c>
       <c r="C138" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D138" s="6"/>
       <c r="E138" s="7" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="F138" s="11" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A139" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B139" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C139" s="6" t="s">
-        <v>101</v>
+        <v>60</v>
       </c>
       <c r="D139" s="6"/>
       <c r="E139" s="7" t="s">
         <v>64</v>
       </c>
       <c r="F139" s="11" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="140" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A140" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B140" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C140" s="6" t="s">
-        <v>59</v>
+        <v>101</v>
       </c>
       <c r="D140" s="6"/>
       <c r="E140" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F140" s="11" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="141" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A141" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B141" s="6" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C141" s="6" t="s">
         <v>59</v>
@@ -3057,15 +3072,15 @@
         <v>63</v>
       </c>
       <c r="F141" s="11" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="142" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A142" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B142" s="6" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="C142" s="6" t="s">
         <v>59</v>
@@ -3075,15 +3090,15 @@
         <v>63</v>
       </c>
       <c r="F142" s="11" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="143" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A143" s="6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B143" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C143" s="6" t="s">
         <v>59</v>
@@ -3093,15 +3108,15 @@
         <v>63</v>
       </c>
       <c r="F143" s="11" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A144" s="6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B144" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C144" s="6" t="s">
         <v>59</v>
@@ -3111,92 +3126,90 @@
         <v>63</v>
       </c>
       <c r="F144" s="11" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A145" s="6">
+        <v>8</v>
+      </c>
+      <c r="B145" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C145" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D145" s="6"/>
+      <c r="E145" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F145" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="G144" s="2">
+      <c r="G145" s="2">
         <v>17</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A146" s="10" t="s">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A147" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B146" s="1" t="s">
+      <c r="B147" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A147" s="10" t="s">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A148" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B147" s="1" t="s">
+      <c r="B148" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A148" s="4" t="s">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A149" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B148" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C148" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D148" s="4" t="s">
+      <c r="B149" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C149" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D149" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E148" s="5" t="s">
+      <c r="E149" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F148" s="5" t="s">
+      <c r="F149" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="149" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A149" s="6">
-        <v>1</v>
-      </c>
-      <c r="B149" s="6" t="s">
+    <row r="150" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A150" s="6">
+        <v>1</v>
+      </c>
+      <c r="B150" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C149" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D149" s="6"/>
-      <c r="E149" s="7" t="s">
+      <c r="C150" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D150" s="6"/>
+      <c r="E150" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="F149" s="11" t="s">
+      <c r="F150" s="11" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A150" s="6">
-        <v>2</v>
-      </c>
-      <c r="B150" s="6" t="s">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A151" s="6">
+        <v>2</v>
+      </c>
+      <c r="B151" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="C150" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="D150" s="6">
-        <v>30</v>
-      </c>
-      <c r="E150" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="F150" s="11" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A151" s="6">
-        <v>3</v>
-      </c>
-      <c r="B151" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="C151" s="6" t="s">
         <v>61</v>
@@ -3208,15 +3221,15 @@
         <v>64</v>
       </c>
       <c r="F151" s="11" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A152" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B152" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C152" s="6" t="s">
         <v>61</v>
@@ -3224,55 +3237,55 @@
       <c r="D152" s="6">
         <v>30</v>
       </c>
-      <c r="E152" s="7"/>
+      <c r="E152" s="7" t="s">
+        <v>64</v>
+      </c>
       <c r="F152" s="11" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A153" s="6">
+        <v>4</v>
+      </c>
+      <c r="B153" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C153" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D153" s="6">
+        <v>30</v>
+      </c>
+      <c r="E153" s="7"/>
+      <c r="F153" s="11" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="153" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A153" s="6">
+    <row r="154" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A154" s="6">
         <v>5</v>
       </c>
-      <c r="B153" s="6" t="s">
+      <c r="B154" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C153" s="6" t="s">
+      <c r="C154" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D153" s="6"/>
-      <c r="E153" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="F153" s="11" t="s">
+      <c r="D154" s="6"/>
+      <c r="E154" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="F154" s="11" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A154" s="6">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A155" s="6">
         <v>6</v>
       </c>
-      <c r="B154" s="6" t="s">
+      <c r="B155" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="C154" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="D154" s="6">
-        <v>20</v>
-      </c>
-      <c r="E154" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="F154" s="11" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A155" s="6">
-        <v>7</v>
-      </c>
-      <c r="B155" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="C155" s="6" t="s">
         <v>61</v>
@@ -3284,27 +3297,47 @@
         <v>64</v>
       </c>
       <c r="F155" s="11" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A156" s="6">
+        <v>7</v>
+      </c>
+      <c r="B156" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C156" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D156" s="6">
+        <v>20</v>
+      </c>
+      <c r="E156" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="F156" s="11" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="156" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A156" s="6">
+    <row r="157" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A157" s="6">
         <v>8</v>
       </c>
-      <c r="B156" s="6" t="s">
+      <c r="B157" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C156" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D156" s="6"/>
-      <c r="E156" s="7" t="s">
+      <c r="C157" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D157" s="6"/>
+      <c r="E157" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="F156" s="11" t="s">
+      <c r="F157" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="G156" s="2">
+      <c r="G157" s="2">
         <v>18</v>
       </c>
     </row>

</xml_diff>